<commit_message>
Added iir filter to script
</commit_message>
<xml_diff>
--- a/modules/iir_filter/iir_filter.xlsx
+++ b/modules/iir_filter/iir_filter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robot\OneDrive\Documents\VHDL\modules\iir_filter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380C8014-A723-4791-9BCD-BBAFFCAC0FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E906D32B-8541-4AE3-9686-7A9CD51397BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2E5E780B-25E9-4007-BA10-822CF03C9BD4}"/>
   </bookViews>
@@ -472,15 +472,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>266701</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>434341</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
-      <xdr:colOff>54009</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>68713</xdr:rowOff>
+      <xdr:colOff>221649</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>53473</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -503,8 +503,52 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6362701" y="7863840"/>
+          <a:off x="6530341" y="7482840"/>
           <a:ext cx="7712108" cy="1531753"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>381001</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>168151</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>145125</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1E999797-A7AD-A544-79FA-80905BBAA26D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6477001" y="8961120"/>
+          <a:ext cx="5883150" cy="3985605"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>